<commit_message>
Hardware: use 10k for R7 so every SMD part is in Robotistan's stock
Robotistan's BOM check reported the 100k part (C17407, an LCSC "(SMT)"
listing) as out of stock. R7 only pulls the unused IO2 input low, so its
value does not matter. It now uses the same 10k part as R2-R6 and the
assembly BOM shrinks to 8 lines. Placement and copper are unchanged.

Also pin the creation time KiCad writes into gerber and drill files to
DATE, so the gerber zip only changes when the board does.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdkdNf8EcXy8Er9VmQyghz
</commit_message>
<xml_diff>
--- a/hardware/kicad/fab/magpanel-carrier-robotistan-bom.xlsx
+++ b/hardware/kicad/fab/magpanel-carrier-robotistan-bom.xlsx
@@ -316,7 +316,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">R2,R3,R4,R5,R6</t>
+          <t xml:space="preserve">R2,R3,R4,R5,R6,R7</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -335,18 +335,18 @@
         </is>
       </c>
       <c r="F8" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">100k 1% SMD Resistor</t>
+          <t xml:space="preserve">33R 1% SMD Resistor</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">R7</t>
+          <t xml:space="preserve">R10,R11,R12,R13,R14,R15,R16,R17,R18,R19,R20,R21,R22,R23,R24,R25</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
@@ -356,45 +356,15 @@
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17407</t>
+          <t xml:space="preserve">C17634</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">0805W8F1003T5E</t>
+          <t xml:space="preserve">0805W8F330JT5E</t>
         </is>
       </c>
       <c r="F9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">33R 1% SMD Resistor</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R10,R11,R12,R13,R14,R15,R16,R17,R18,R19,R20,R21,R22,R23,R24,R25</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0805</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C17634</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0805W8F330JT5E</t>
-        </is>
-      </c>
-      <c r="F10" s="1">
         <v>16</v>
       </c>
     </row>

</xml_diff>